<commit_message>
Re-estimate the fifty companies on the Australian DIA rates
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated. The register held through the
run - 29 approved, 25 revoked, 5 undecided - and research challenged
seven decisions with other figures, 21 times, which the card did not
take.

The set baseline moves from EUR 566,093,106 to 565,580,455 (-0.51M), all
of it Woolworths: AUD 8.95m to 8.08m (-9.7%), its 30 primary 100 Mbps DIA
circuits moving from the AUD 2,072 300 Mbps seed to the approved AUD 339
and its four 500 Mbps backups to the sourced 484. Best-case saving falls
EUR 0.14M to 112.1M; Woolworths' steady-state payback goes from 17 months
to 19. Sourced prices now carry 26.7% of priced value. The other 49
companies change only in run ids and timestamps; 49 stay COMPLETE for
their declared scope and Capgemini PARTIAL, as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/price-review.xlsx
+++ b/docs/price-review.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Every researched price on the rate card - 28 approved, 25 revoked, 6 undecided - beside the rate it would replace, with its evidence and what its approval does to the sample baselines.</t>
+          <t>Every researched price on the rate card - 29 approved, 25 revoked, 5 undecided - beside the rate it would replace, with its evidence and what its approval does to the sample baselines.</t>
         </is>
       </c>
     </row>
@@ -789,21 +789,21 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>AU-DIA-250-researched</t>
+          <t>BE-BROADBAND_PON-2500-researched</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>BROADBAND_PON</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>250</v>
+        <v>2500</v>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
@@ -817,7 +817,7 @@
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Vocus publishes Fast Fibre from A$339/month ex GST. Hold because it is a floor and the same research cites materially higher enterprise dedicated-fibre ranges.</t>
+          <t>Proximus Flex+ is a small-business pack 'from' EUR 95 with services bundled in, not a connectivity price. No circuit in the set uses it.</t>
         </is>
       </c>
       <c r="H2" s="9">
@@ -829,15 +829,15 @@
         <v/>
       </c>
       <c r="J2" s="10" t="n">
-        <v>339</v>
+        <v>95</v>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>AUD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="L2" s="10" t="n">
-        <v>229.05</v>
+        <v>109.06</v>
       </c>
       <c r="M2" s="10" t="n"/>
       <c r="N2" s="11">
@@ -851,67 +851,75 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>single source</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr"/>
+          <t>floor; single source; re-prices lower tiers</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>BROADBAND_PON 2500 Mbps MRC (Proximus Flex+ Giga Fiber 2.5 Gbps)</t>
+        </is>
+      </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>run narrative (the disposition was replaced)</t>
+          <t>Proximus (proximus.com press release Jul 2025); COMPANY_PUBLISHED/FULL_PAGE</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>advertised price ~A$65-80/mo (not enterprise). AU DIA (Dedicated Internet Access – direct fibre): Nexthop AU lists 1 Gbps datacenter DIA at A$499/mo (24-month, on-net); Vocus Fast Fibre (direct fibre, enterprise) from A$339/mo excl. GST for 250 Mbps+. AyeTech 2026 guide cites enterprise dedicated fibre 100 Mbps–1 Gbps at A$2,500–A$8,000/mo for large-enterprise/data-centre grade. N</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="inlineStr"/>
+          <t>Business Flex+ Giga Fiber 2.5 Gbps symmetric: from €95/month</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proximus.com/news/2025/202507-business-flex-plus-packs-as-of-july-1-2025.html</t>
+        </is>
+      </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>woolworths</t>
+          <t>bnp-paribas</t>
         </is>
       </c>
       <c r="W2" s="12" t="n">
-        <v>-459004.9560810811</v>
+        <v>0</v>
       </c>
       <c r="X2" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="Y2" s="3" t="inlineStr">
-        <is>
-          <t>woolworths -459,005</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y2" s="3" t="inlineStr"/>
       <c r="Z2" s="3" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA2" s="3" t="inlineStr"/>
+          <t>1000 Mbps at 136 &gt; 2500 Mbps at 109 USD</t>
+        </is>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>bnp-paribas 95 EUR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>BE-BROADBAND_PON-2500-researched</t>
+          <t>ES-DIA-100-researched</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>BROADBAND_PON</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>2500</v>
+        <v>100</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
@@ -925,7 +933,7 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Proximus Flex+ is a small-business pack 'from' EUR 95 with services bundled in, not a connectivity price. No circuit in the set uses it.</t>
+          <t>Held: Direct Telecom's EUR 159.99 is a guaranteed rather than dedicated circuit, below Kompara's EUR 200-300 for 100 Mbps dedicated fibre. The card now prices Spain DIA 100 at that range's EUR 250 midpoint as a sourced rate; approving this row would displace it.</t>
         </is>
       </c>
       <c r="H3" s="9">
@@ -937,7 +945,7 @@
         <v/>
       </c>
       <c r="J3" s="10" t="n">
-        <v>95</v>
+        <v>159.99</v>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
@@ -945,80 +953,74 @@
         </is>
       </c>
       <c r="L3" s="10" t="n">
-        <v>109.06</v>
-      </c>
-      <c r="M3" s="10" t="n"/>
+        <v>183.66</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>287</v>
+      </c>
       <c r="N3" s="11">
         <f>IF(OR(L3="",M3=""),"",L3/M3)</f>
         <v/>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>none - new tier</t>
+          <t>SEED</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>floor; single source; re-prices lower tiers</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>BROADBAND_PON 2500 Mbps MRC (Proximus Flex+ Giga Fiber 2.5 Gbps)</t>
-        </is>
-      </c>
+          <t>single source</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr"/>
       <c r="R3" s="5" t="inlineStr">
         <is>
-          <t>Proximus (proximus.com press release Jul 2025); COMPANY_PUBLISHED/FULL_PAGE</t>
+          <t>run narrative (the disposition was replaced)</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>Business Flex+ Giga Fiber 2.5 Gbps symmetric: from €95/month</t>
-        </is>
-      </c>
-      <c r="T3" s="5" t="inlineStr">
-        <is>
-          <t>https://www.proximus.com/news/2025/202507-business-flex-plus-packs-as-of-july-1-2025.html</t>
-        </is>
-      </c>
+          <t>band, MPLS/IP-VPN and SD-WAN from all four national players plus resellers. Telefónica Global Solutions offers DIA on its own Tier 1 global infrastructure. A domestic reseller (Direct Telecom) lists 100/100 Mbps DIA at €159.99/month and 1 Gbps dedicated circuit at €449/month (2025 prices). Telefónica and MasOrange are exploring acquisition of Vodafone España (as of mid-2025); if comp</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr"/>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>bnp-paribas</t>
+          <t>inditex</t>
         </is>
       </c>
       <c r="W3" s="12" t="n">
-        <v>0</v>
+        <v>-2357511.18</v>
       </c>
       <c r="X3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="3" t="inlineStr"/>
+        <v>2072</v>
+      </c>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>santander -1,760,707; fresenius -580,601; carrefour -16,203</t>
+        </is>
+      </c>
       <c r="Z3" s="3" t="inlineStr">
         <is>
-          <t>1000 Mbps at 136 &gt; 2500 Mbps at 109 USD</t>
-        </is>
-      </c>
-      <c r="AA3" s="3" t="inlineStr">
-        <is>
-          <t>bnp-paribas 95 EUR</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>ES-DIA-100-researched</t>
+          <t>SG-DIA-100-researched</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -1041,7 +1043,7 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>Held: Direct Telecom's EUR 159.99 is a guaranteed rather than dedicated circuit, below Kompara's EUR 200-300 for 100 Mbps dedicated fibre. The card now prices Spain DIA 100 at that range's EUR 250 midpoint as a sourced rate; approving this row would displace it.</t>
+          <t>Published on SPTel's promotion page (valid to 31 Dec 2026). No circuit in the set uses it.</t>
         </is>
       </c>
       <c r="H4" s="9">
@@ -1053,18 +1055,18 @@
         <v/>
       </c>
       <c r="J4" s="10" t="n">
-        <v>159.99</v>
+        <v>312</v>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="L4" s="10" t="n">
-        <v>183.66</v>
+        <v>243.75</v>
       </c>
       <c r="M4" s="10" t="n">
-        <v>287</v>
+        <v>660</v>
       </c>
       <c r="N4" s="11">
         <f>IF(OR(L4="",M4=""),"",L4/M4)</f>
@@ -1077,67 +1079,75 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>single source</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr"/>
+          <t>single source; read from a snippet</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>DIA 100 Mbps MRC — Singapore (SPTel enterprise tariff)</t>
+        </is>
+      </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>run narrative (the disposition was replaced)</t>
+          <t>SPTel; COMPANY_PUBLISHED/SNIPPET_ONLY</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>band, MPLS/IP-VPN and SD-WAN from all four national players plus resellers. Telefónica Global Solutions offers DIA on its own Tier 1 global infrastructure. A domestic reseller (Direct Telecom) lists 100/100 Mbps DIA at €159.99/month and 1 Gbps dedicated circuit at €449/month (2025 prices). Telefónica and MasOrange are exploring acquisition of Vodafone España (as of mid-2025); if comp</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr"/>
+          <t>Enterprise Internet 100Mbps $312/mth (on 24-month contract)</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>https://sptel.com/promotion/business-broadband-singapore/</t>
+        </is>
+      </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>inditex</t>
+          <t>dbs</t>
         </is>
       </c>
       <c r="W4" s="12" t="n">
-        <v>-2357511.18</v>
+        <v>0</v>
       </c>
       <c r="X4" s="5" t="n">
-        <v>2072</v>
-      </c>
-      <c r="Y4" s="3" t="inlineStr">
-        <is>
-          <t>santander -1,760,707; fresenius -580,601; carrefour -16,203</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y4" s="3" t="inlineStr"/>
       <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AA4" s="3" t="inlineStr"/>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>dbs 312 SGD; dbs 312 SGD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>SG-DIA-100-researched</t>
+          <t>US-BROADBAND_PON-300-researched</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>BROADBAND_PON</t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -1151,7 +1161,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Published on SPTel's promotion page (valid to 31 Dec 2026). No circuit in the set uses it.</t>
+          <t>AT&amp;T Business Fiber 300, inside AT&amp;T's footprint only. At $70 it is below the national median for 100 Mbps, and would price every US PON circuit up to 300 Mbps at it.</t>
         </is>
       </c>
       <c r="H5" s="9">
@@ -1163,51 +1173,49 @@
         <v/>
       </c>
       <c r="J5" s="10" t="n">
-        <v>312</v>
+        <v>70</v>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L5" s="10" t="n">
-        <v>243.75</v>
-      </c>
-      <c r="M5" s="10" t="n">
-        <v>660</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="M5" s="10" t="n"/>
       <c r="N5" s="11">
         <f>IF(OR(L5="",M5=""),"",L5/M5)</f>
         <v/>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>SEED</t>
+          <t>none - new tier</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>single source; read from a snippet</t>
+          <t>read from a snippet; re-prices lower tiers</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>DIA 100 Mbps MRC — Singapore (SPTel enterprise tariff)</t>
+          <t>BROADBAND_PON 300 Mbps MRC – US (AT&amp;T Business Fiber published rate)</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>SPTel; COMPANY_PUBLISHED/SNIPPET_ONLY</t>
+          <t>business.org (AT&amp;T Business Internet Review 2026); AGGREGATOR/SNIPPET_ONLY</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>Enterprise Internet 100Mbps $312/mth (on 24-month contract)</t>
+          <t>Business Fiber 300: $70.00/mo</t>
         </is>
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>https://sptel.com/promotion/business-broadband-singapore/</t>
+          <t>https://www.business.org/services/internet/att-business-internet-review/</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
@@ -1217,45 +1225,49 @@
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>dbs</t>
+          <t>simmons-bank</t>
         </is>
       </c>
       <c r="W5" s="12" t="n">
-        <v>0</v>
+        <v>-75873.6111235</v>
       </c>
       <c r="X5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="3" t="inlineStr"/>
+        <v>243</v>
+      </c>
+      <c r="Y5" s="3" t="inlineStr">
+        <is>
+          <t>simmons-bank -39,654; basf -8,430; siemens -7,181</t>
+        </is>
+      </c>
       <c r="Z5" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>250 Mbps at 114 &gt; 300 Mbps at 70 USD</t>
         </is>
       </c>
       <c r="AA5" s="3" t="inlineStr">
         <is>
-          <t>dbs 312 SGD; dbs 312 SGD</t>
+          <t>simmons-bank 70 USD</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>US-BROADBAND_PON-300-researched</t>
+          <t>ZA-DIA-100-researched</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ZA</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BROADBAND_PON</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -1269,7 +1281,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>AT&amp;T Business Fiber 300, inside AT&amp;T's footprint only. At $70 it is below the national median for 100 Mbps, and would price every US PON circuit up to 300 Mbps at it.</t>
+          <t>MWCom 'from around R8,000'; the same research gives R8,000-25,000 depending on distance and capacity.</t>
         </is>
       </c>
       <c r="H6" s="9">
@@ -1281,15 +1293,15 @@
         <v/>
       </c>
       <c r="J6" s="10" t="n">
-        <v>70</v>
+        <v>8000</v>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>ZAR</t>
         </is>
       </c>
       <c r="L6" s="10" t="n">
-        <v>70</v>
+        <v>444.44</v>
       </c>
       <c r="M6" s="10" t="n"/>
       <c r="N6" s="11">
@@ -1303,27 +1315,27 @@
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>read from a snippet; re-prices lower tiers</t>
+          <t>floor; read from a snippet</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>BROADBAND_PON 300 Mbps MRC – US (AT&amp;T Business Fiber published rate)</t>
+          <t>DIA 100 Mbps MRC ZA (leased line / dedicated fibre)</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>business.org (AT&amp;T Business Internet Review 2026); AGGREGATOR/SNIPPET_ONLY</t>
+          <t>mwcom.co.za; COMPANY_PUBLISHED/SNIPPET_ONLY</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>Business Fiber 300: $70.00/mo</t>
+          <t>Leased lines start from around R8,000/mo for 100 Mbps symmetric.</t>
         </is>
       </c>
       <c r="T6" s="5" t="inlineStr">
         <is>
-          <t>https://www.business.org/services/internet/att-business-internet-review/</t>
+          <t>https://www.mwcom.co.za/business-internet-south-africa</t>
         </is>
       </c>
       <c r="U6" s="5" t="inlineStr">
@@ -1333,63 +1345,59 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>simmons-bank</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="W6" s="12" t="n">
-        <v>-75873.6111235</v>
+        <v>-16474.2432</v>
       </c>
       <c r="X6" s="5" t="n">
-        <v>243</v>
+        <v>1</v>
       </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>simmons-bank -39,654; basf -8,430; siemens -7,181</t>
+          <t>anglo-american -16,474</t>
         </is>
       </c>
       <c r="Z6" s="3" t="inlineStr">
         <is>
-          <t>250 Mbps at 114 &gt; 300 Mbps at 70 USD</t>
-        </is>
-      </c>
-      <c r="AA6" s="3" t="inlineStr">
-        <is>
-          <t>simmons-bank 70 USD</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>ZA-DIA-100-researched</t>
+          <t>AU-BROADBAND_HFC-250-researched</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ZA</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>BROADBAND_HFC</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>undecided</t>
+        <v>250</v>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>approved by Christian Bartosch</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Approve</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>MWCom 'from around R8,000'; the same research gives R8,000-25,000 depending on distance and capacity.</t>
+          <t>Swoop's published standard business nbn 250/100 price of A$104/month. The introductory discount is excluded.</t>
         </is>
       </c>
       <c r="H7" s="9">
@@ -1401,75 +1409,69 @@
         <v/>
       </c>
       <c r="J7" s="10" t="n">
-        <v>8000</v>
+        <v>104</v>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>ZAR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="L7" s="10" t="n">
-        <v>444.44</v>
-      </c>
-      <c r="M7" s="10" t="n"/>
+        <v>70.27</v>
+      </c>
+      <c r="M7" s="10" t="n">
+        <v>155</v>
+      </c>
       <c r="N7" s="11">
         <f>IF(OR(L7="",M7=""),"",L7/M7)</f>
         <v/>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>none - new tier</t>
+          <t>SEED</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>floor; read from a snippet</t>
-        </is>
-      </c>
-      <c r="Q7" s="3" t="inlineStr">
-        <is>
-          <t>DIA 100 Mbps MRC ZA (leased line / dedicated fibre)</t>
-        </is>
-      </c>
+          <t>single source; re-prices lower tiers</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr"/>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>mwcom.co.za; COMPANY_PUBLISHED/SNIPPET_ONLY</t>
+          <t>run narrative (the disposition was replaced)</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>Leased lines start from around R8,000/mo for 100 Mbps symmetric.</t>
-        </is>
-      </c>
-      <c r="T7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.mwcom.co.za/business-internet-south-africa</t>
-        </is>
-      </c>
+          <t>ise NBN (symmetric, SLA-backed) list prices in AUD excl. GST: 100/100 Mbps A$399/mo, 250/250 Mbps A$399/mo, 500/500 Mbps A$469/mo, 1000/1000 Mbps A$699/mo (36-month term). Swoop published business NBN prices: 250 Mbps A$104/mo (FTTP), 1000 Mbps A$129/mo (FTTP/HFC). Kookaburra Comms (trade press, 2026) cites typical published range A$400 for 100-250 Mbps to A$700-A$1,500 for 1 Gbps</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr"/>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>not recorded</t>
+          <t>woolworths</t>
         </is>
       </c>
       <c r="W7" s="12" t="n">
-        <v>-16474.2432</v>
+        <v>-925814.4972972973</v>
       </c>
       <c r="X7" s="5" t="n">
-        <v>1</v>
+        <v>1130</v>
       </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>anglo-american -16,474</t>
+          <t>woolworths -925,814</t>
         </is>
       </c>
       <c r="Z7" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>100 Mbps at 115 &gt; 250 Mbps at 70 USD; 1000 Mbps at 250 &gt; 2000 Mbps at 149 USD</t>
         </is>
       </c>
       <c r="AA7" s="3" t="inlineStr"/>
@@ -1477,7 +1479,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>AU-BROADBAND_HFC-250-researched</t>
+          <t>AU-BROADBAND_HFC-2000-researched</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1491,7 +1493,7 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>250</v>
+        <v>2000</v>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
@@ -1505,7 +1507,7 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Swoop's published standard business nbn 250/100 price of A$104/month. The introductory discount is excluded.</t>
+          <t>Aussie Broadband business Hyperfast 2000, published; a trade guide puts business fibre plans at A$100-220.</t>
         </is>
       </c>
       <c r="H8" s="9">
@@ -1517,7 +1519,7 @@
         <v/>
       </c>
       <c r="J8" s="10" t="n">
-        <v>104</v>
+        <v>220</v>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
@@ -1525,40 +1527,46 @@
         </is>
       </c>
       <c r="L8" s="10" t="n">
-        <v>70.27</v>
-      </c>
-      <c r="M8" s="10" t="n">
-        <v>155</v>
-      </c>
+        <v>148.65</v>
+      </c>
+      <c r="M8" s="10" t="n"/>
       <c r="N8" s="11">
         <f>IF(OR(L8="",M8=""),"",L8/M8)</f>
         <v/>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>SEED</t>
+          <t>none - new tier</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>single source; re-prices lower tiers</t>
-        </is>
-      </c>
-      <c r="Q8" s="3" t="inlineStr"/>
+          <t>read from a snippet; re-prices lower tiers</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>BROADBAND_HFC AU 2000Mbps MRC (Aussie Broadband Business Hyperfast HFC)</t>
+        </is>
+      </c>
       <c r="R8" s="5" t="inlineStr">
         <is>
-          <t>run narrative (the disposition was replaced)</t>
+          <t>Aussie Broadband / WhistleOut; AGGREGATOR/SNIPPET_ONLY</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>ise NBN (symmetric, SLA-backed) list prices in AUD excl. GST: 100/100 Mbps A$399/mo, 250/250 Mbps A$399/mo, 500/500 Mbps A$469/mo, 1000/1000 Mbps A$699/mo (36-month term). Swoop published business NBN prices: 250 Mbps A$104/mo (FTTP), 1000 Mbps A$129/mo (FTTP/HFC). Kookaburra Comms (trade press, 2026) cites typical published range A$400 for 100-250 Mbps to A$700-A$1,500 for 1 Gbps</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr"/>
+          <t>Aussie Broadband FTTP Business Hyperfast Plus 2000/500 Unlimited Data $220/mth</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.whistleout.com.au/Broadband/Guides/NBN-business-plans-compared</t>
+        </is>
+      </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
@@ -1567,27 +1575,27 @@
         </is>
       </c>
       <c r="W8" s="12" t="n">
-        <v>-925814.4972972973</v>
+        <v>0</v>
       </c>
       <c r="X8" s="5" t="n">
-        <v>1130</v>
-      </c>
-      <c r="Y8" s="3" t="inlineStr">
-        <is>
-          <t>woolworths -925,814</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="3" t="inlineStr"/>
       <c r="Z8" s="3" t="inlineStr">
         <is>
           <t>100 Mbps at 115 &gt; 250 Mbps at 70 USD; 1000 Mbps at 250 &gt; 2000 Mbps at 149 USD</t>
         </is>
       </c>
-      <c r="AA8" s="3" t="inlineStr"/>
+      <c r="AA8" s="3" t="inlineStr">
+        <is>
+          <t>woolworths 220 AUD</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>AU-BROADBAND_HFC-2000-researched</t>
+          <t>AU-BROADBAND_PON-250-researched</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1597,11 +1605,11 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>BROADBAND_HFC</t>
+          <t>BROADBAND_PON</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>2000</v>
+        <v>250</v>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
@@ -1615,7 +1623,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Aussie Broadband business Hyperfast 2000, published; a trade guide puts business fibre plans at A$100-220.</t>
+          <t>Aussie Broadband business FTTP 250/100, published by the provider and confirmed by an aggregator.</t>
         </is>
       </c>
       <c r="H9" s="9">
@@ -1627,7 +1635,7 @@
         <v/>
       </c>
       <c r="J9" s="10" t="n">
-        <v>220</v>
+        <v>114</v>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
@@ -1635,41 +1643,43 @@
         </is>
       </c>
       <c r="L9" s="10" t="n">
-        <v>148.65</v>
-      </c>
-      <c r="M9" s="10" t="n"/>
+        <v>77.03</v>
+      </c>
+      <c r="M9" s="10" t="n">
+        <v>101</v>
+      </c>
       <c r="N9" s="11">
         <f>IF(OR(L9="",M9=""),"",L9/M9)</f>
         <v/>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>none - new tier</t>
+          <t>SEED</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>read from a snippet; re-prices lower tiers</t>
+          <t>read from a snippet</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>BROADBAND_HFC AU 2000Mbps MRC (Aussie Broadband Business Hyperfast HFC)</t>
+          <t>BROADBAND_PON AU 250Mbps MRC (Aussie Broadband Business FTTP 250/100)</t>
         </is>
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Aussie Broadband / WhistleOut; AGGREGATOR/SNIPPET_ONLY</t>
+          <t>Aussie Broadband Enterprise; COMPANY_PUBLISHED/SNIPPET_ONLY</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>Aussie Broadband FTTP Business Hyperfast Plus 2000/500 Unlimited Data $220/mth</t>
+          <t>Superfast Plus 250/100 $114/month</t>
         </is>
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>https://www.whistleout.com.au/Broadband/Guides/NBN-business-plans-compared</t>
+          <t>https://www.aussiebroadband.com.au/enterprise/internet/nbn-plans/</t>
         </is>
       </c>
       <c r="U9" s="5" t="inlineStr">
@@ -1691,19 +1701,19 @@
       <c r="Y9" s="3" t="inlineStr"/>
       <c r="Z9" s="3" t="inlineStr">
         <is>
-          <t>100 Mbps at 115 &gt; 250 Mbps at 70 USD; 1000 Mbps at 250 &gt; 2000 Mbps at 149 USD</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AA9" s="3" t="inlineStr">
         <is>
-          <t>woolworths 220 AUD</t>
+          <t>woolworths 114 AUD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>AU-BROADBAND_PON-250-researched</t>
+          <t>AU-DIA-250-researched</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1713,7 +1723,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>BROADBAND_PON</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
@@ -1731,19 +1741,17 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Aussie Broadband business FTTP 250/100, published by the provider and confirmed by an aggregator.</t>
-        </is>
-      </c>
-      <c r="H10" s="9">
-        <f>J10*0.75</f>
-        <v/>
-      </c>
-      <c r="I10" s="9">
-        <f>J10*1.25</f>
-        <v/>
+          <t>Vocus Fast Fibre 250/250: dedicated 1:1 fibre with internet, a static IP and a 4-hour restoration SLA, at its on-net 48-month price ex GST. Second sources sit within 18%: Telair resells it at A$349 on 36 months, and Vocus and Swoop sell 250/250 nbn Enterprise Ethernet at A$399. The band runs from the 48-month price to the 36-month Enterprise Ethernet one. The A$2,500-8,000 in the same research is data-centre-grade carrier fibre, which no seller publishes.</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>339</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>399</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>114</v>
+        <v>339</v>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
@@ -1751,48 +1759,38 @@
         </is>
       </c>
       <c r="L10" s="10" t="n">
-        <v>77.03</v>
-      </c>
-      <c r="M10" s="10" t="n">
-        <v>101</v>
-      </c>
+        <v>229.05</v>
+      </c>
+      <c r="M10" s="10" t="n"/>
       <c r="N10" s="11">
         <f>IF(OR(L10="",M10=""),"",L10/M10)</f>
         <v/>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>SEED</t>
+          <t>none - new tier</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>read from a snippet</t>
-        </is>
-      </c>
-      <c r="Q10" s="3" t="inlineStr">
-        <is>
-          <t>BROADBAND_PON AU 250Mbps MRC (Aussie Broadband Business FTTP 250/100)</t>
-        </is>
-      </c>
+          <t>single source</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>Aussie Broadband Enterprise; COMPANY_PUBLISHED/SNIPPET_ONLY</t>
+          <t>run narrative (the disposition was replaced)</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>Superfast Plus 250/100 $114/month</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.aussiebroadband.com.au/enterprise/internet/nbn-plans/</t>
-        </is>
-      </c>
+          <t>advertised price ~A$65-80/mo (not enterprise). AU DIA (Dedicated Internet Access – direct fibre): Nexthop AU lists 1 Gbps datacenter DIA at A$499/mo (24-month, on-net); Vocus Fast Fibre (direct fibre, enterprise) from A$339/mo excl. GST for 250 Mbps+. AyeTech 2026 guide cites enterprise dedicated fibre 100 Mbps–1 Gbps at A$2,500–A$8,000/mo for large-enterprise/data-centre grade. N</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr"/>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
@@ -1801,22 +1799,22 @@
         </is>
       </c>
       <c r="W10" s="12" t="n">
-        <v>0</v>
+        <v>-21538.53608108108</v>
       </c>
       <c r="X10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="3" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="Y10" s="3" t="inlineStr">
+        <is>
+          <t>woolworths -21,539</t>
+        </is>
+      </c>
       <c r="Z10" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AA10" s="3" t="inlineStr">
-        <is>
-          <t>woolworths 114 AUD</t>
-        </is>
-      </c>
+      <c r="AA10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -4820,7 +4818,7 @@
         <v>337.16</v>
       </c>
       <c r="M36" s="10" t="n">
-        <v>1750</v>
+        <v>742</v>
       </c>
       <c r="N36" s="11">
         <f>IF(OR(L36="",M36=""),"",L36/M36)</f>
@@ -4833,7 +4831,7 @@
       </c>
       <c r="P36" s="3" t="inlineStr">
         <is>
-          <t>consumer; single source; re-prices lower tiers</t>
+          <t>consumer; single source</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr"/>
@@ -4859,19 +4857,15 @@
         </is>
       </c>
       <c r="W36" s="12" t="n">
-        <v>-416627.1182432433</v>
+        <v>0</v>
       </c>
       <c r="X36" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="Y36" s="3" t="inlineStr">
-        <is>
-          <t>woolworths -416,627</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y36" s="3" t="inlineStr"/>
       <c r="Z36" s="3" t="inlineStr">
         <is>
-          <t>500 Mbps at 1610 &gt; 1000 Mbps at 337 USD</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AA36" s="3" t="inlineStr"/>
@@ -7783,19 +7777,19 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
       <c r="E4" s="16" t="n">
-        <v>0</v>
+        <v>-21538.53608108108</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>-459004.9560810811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -8620,17 +8614,17 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>5269388.71</v>
+        <v>4756737.94</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>-1054065.373135135</v>
+        <v>-1075603.909216216</v>
       </c>
       <c r="D6" s="19">
         <f>IF(B6=0,"",C6/B6)</f>
         <v/>
       </c>
       <c r="E6" s="16" t="n">
-        <v>-459004.9560810811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -9276,11 +9270,11 @@
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>anglo-american</t>
+          <t>carrefour</t>
         </is>
       </c>
       <c r="B39" s="16" t="n">
-        <v>373694.9</v>
+        <v>39782444.83</v>
       </c>
       <c r="C39" s="16" t="n">
         <v>0</v>
@@ -9290,17 +9284,17 @@
         <v/>
       </c>
       <c r="E39" s="16" t="n">
-        <v>-16474.2432</v>
+        <v>-16202.83</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>carrefour</t>
+          <t>anglo-american</t>
         </is>
       </c>
       <c r="B40" s="16" t="n">
-        <v>39782444.83</v>
+        <v>373694.9</v>
       </c>
       <c r="C40" s="16" t="n">
         <v>0</v>
@@ -9310,7 +9304,7 @@
         <v/>
       </c>
       <c r="E40" s="16" t="n">
-        <v>-16202.83</v>
+        <v>-16474.2432</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
Re-estimate the fifty companies with UK DIA at 10 Gbps
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated. The register held through the
run, and research challenged seven decisions with other figures, 21
times, which the card did not take.

The set baseline moves from EUR 574,105,804 to 577,434,188 (+3.3M,
+0.6%), exactly what was priced before the change, across the five
companies whose 10 Gbps DIA backups had no rate: Capgemini +1.7M
(+30.9%), Allianz +1.0M, Generali +0.3M, Fraport +0.2M, Aena +0.1M. 111
circuits are newly priced, 102 of them at the regional rate outside the
UK. Allianz, Generali, Fraport and Aena now price every circuit;
Capgemini reaches 96.0% of spend and stays PARTIAL on its 19 Indian DIA
backups. Best-case saving rises EUR 0.9M to 115.3M.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/price-review.xlsx
+++ b/docs/price-review.xlsx
@@ -6559,14 +6559,16 @@
       <c r="L51" s="10" t="n">
         <v>602.97</v>
       </c>
-      <c r="M51" s="10" t="n"/>
+      <c r="M51" s="10" t="n">
+        <v>2881</v>
+      </c>
       <c r="N51" s="11">
         <f>IF(OR(L51="",M51=""),"",L51/M51)</f>
         <v/>
       </c>
       <c r="O51" s="5" t="inlineStr">
         <is>
-          <t>none - new tier</t>
+          <t>SEED</t>
         </is>
       </c>
       <c r="P51" s="3" t="inlineStr">
@@ -6605,19 +6607,19 @@
         </is>
       </c>
       <c r="W51" s="12" t="n">
-        <v>56727.13</v>
+        <v>-214313.89</v>
       </c>
       <c r="X51" s="5" t="n">
         <v>9</v>
       </c>
       <c r="Y51" s="3" t="inlineStr">
         <is>
-          <t>capgemini +56,727</t>
+          <t>capgemini -214,314</t>
         </is>
       </c>
       <c r="Z51" s="3" t="inlineStr">
         <is>
-          <t>1000 Mbps at 737 &gt; 10000 Mbps at 603 USD</t>
+          <t>9000 Mbps at 2707 &gt; 10000 Mbps at 603 USD</t>
         </is>
       </c>
       <c r="AA51" s="3" t="inlineStr">
@@ -9210,11 +9212,11 @@
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>anglo-american</t>
+          <t>carrefour</t>
         </is>
       </c>
       <c r="B36" s="16" t="n">
-        <v>373694.9</v>
+        <v>39782444.83</v>
       </c>
       <c r="C36" s="16" t="n">
         <v>0</v>
@@ -9224,17 +9226,17 @@
         <v/>
       </c>
       <c r="E36" s="16" t="n">
-        <v>-16474.2432</v>
+        <v>-16202.83</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>carrefour</t>
+          <t>anglo-american</t>
         </is>
       </c>
       <c r="B37" s="16" t="n">
-        <v>39782444.83</v>
+        <v>373694.9</v>
       </c>
       <c r="C37" s="16" t="n">
         <v>0</v>
@@ -9244,7 +9246,7 @@
         <v/>
       </c>
       <c r="E37" s="16" t="n">
-        <v>-16202.83</v>
+        <v>-16474.2432</v>
       </c>
     </row>
     <row r="38">
@@ -9294,7 +9296,7 @@
         </is>
       </c>
       <c r="B40" s="16" t="n">
-        <v>5548150.74</v>
+        <v>7264743.88</v>
       </c>
       <c r="C40" s="16" t="n">
         <v>112841.25</v>

</xml_diff>

<commit_message>
Re-estimate the fifty companies on Telstra's 5G prices
No provider calls: findings already paid for were re-offered, then each
company re-simulated and re-estimated. The register held through the
run, and research challenged seven decisions with other figures, 21
times, which the card did not take.

The set baseline moves from EUR 577,434,188 to 577,243,208 (-0.19M)
across two companies: Woolworths AUD -285k (-3.5%), its Australian 5G
now at Telstra's rates and its 71 New Zealand backups at APAC's
re-placed 100 Mbps rate, its regionally priced share falling from 20.1%
to 2.1%; and Rio Tinto USD -26k. Best-case saving falls EUR 0.05M to
115.3M. The other 48 companies change only in run ids and timestamps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/price-review.xlsx
+++ b/docs/price-review.xlsx
@@ -8616,7 +8616,7 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>4756737.94</v>
+        <v>4588807.28</v>
       </c>
       <c r="C6" s="16" t="n">
         <v>-1075603.909216216</v>
@@ -8716,7 +8716,7 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>1330261.85</v>
+        <v>1307212.55</v>
       </c>
       <c r="C11" s="16" t="n">
         <v>-304559.635439</v>

</xml_diff>